<commit_message>
Fixed numbering of modules. Added lecture.
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Dropbox/SPS Dropbox/Jason Bryer/Teaching/IS381 2026 Fall/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FE9B0A-AA09-CB44-B6C2-E960071ACB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B844C0-F3CD-FB49-A8D4-3EE67421C0B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1220" yWindow="13680" windowWidth="24780" windowHeight="13780" xr2:uid="{BFE2A6F7-E8E8-014E-9460-2468D969C60C}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>Week</t>
   </si>
@@ -95,39 +95,6 @@
     <t>/assignments/02_R_Coding_Basics.zip</t>
   </si>
   <si>
-    <t>/assignments/04_Data_Visualization.zip</t>
-  </si>
-  <si>
-    <t>/assignments/05_Reshaping_Data.zip</t>
-  </si>
-  <si>
-    <t>/assignments/06_Probability.zip</t>
-  </si>
-  <si>
-    <t>/assignments/07_Distributions.zip</t>
-  </si>
-  <si>
-    <t>/assignments/08_Sampling_Distributions.zip</t>
-  </si>
-  <si>
-    <t>/assignments/09_Confidence_Intervals.zip</t>
-  </si>
-  <si>
-    <t>/assignments/10_Inference_for_Categorical_Data.zip</t>
-  </si>
-  <si>
-    <t>/assignments/11_Chi_Squared.zip</t>
-  </si>
-  <si>
-    <t>/assignments/12_Inference_for_Numerical_Data.zip</t>
-  </si>
-  <si>
-    <t>/assignments/13_ANOVA.zip</t>
-  </si>
-  <si>
-    <t>/assignments/14_Correlation.zip</t>
-  </si>
-  <si>
     <t>/modules/01-Module.html</t>
   </si>
   <si>
@@ -170,9 +137,6 @@
     <t>Reshaping Data</t>
   </si>
   <si>
-    <t>/modules/15-Module.html</t>
-  </si>
-  <si>
     <t>Resources</t>
   </si>
   <si>
@@ -204,6 +168,48 @@
   </si>
   <si>
     <t>ofow-rwsCqY</t>
+  </si>
+  <si>
+    <t>a0KLUwNPkMk</t>
+  </si>
+  <si>
+    <t>03-Data_Visualization</t>
+  </si>
+  <si>
+    <t>/assignments/03_Data_Visualization.zip</t>
+  </si>
+  <si>
+    <t>/assignments/04_Reshaping_Data.zip</t>
+  </si>
+  <si>
+    <t>/assignments/05_Probability.zip</t>
+  </si>
+  <si>
+    <t>/assignments/06_Distributions.zip</t>
+  </si>
+  <si>
+    <t>/assignments/07_Sampling_Distributions.zip</t>
+  </si>
+  <si>
+    <t>/assignments/08_Confidence_Intervals.zip</t>
+  </si>
+  <si>
+    <t>/assignments/09_Inference_for_Categorical_Data.zip</t>
+  </si>
+  <si>
+    <t>/assignments/10_Chi_Squared.zip</t>
+  </si>
+  <si>
+    <t>/assignments/11_Inference_for_Numerical_Data.zip</t>
+  </si>
+  <si>
+    <t>/assignments/12_ANOVA.zip</t>
+  </si>
+  <si>
+    <t>/assignments/13_Correlation.zip</t>
+  </si>
+  <si>
+    <t>/modules/03-Module.html</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1121,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
         <v>17</v>
@@ -1133,7 +1139,7 @@
         <v>13</v>
       </c>
       <c r="J1" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -1152,19 +1158,19 @@
         <v>46265</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G2" t="s">
         <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="I2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -1184,19 +1190,19 @@
         <v>46272</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="G3" t="s">
         <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -1219,10 +1225,16 @@
         <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G4" t="s">
-        <v>20</v>
+        <v>47</v>
+      </c>
+      <c r="H4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -1242,13 +1254,13 @@
         <v>46286</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -1271,10 +1283,10 @@
         <v>15</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -1297,10 +1309,10 @@
         <v>16</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1323,10 +1335,10 @@
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -1346,13 +1358,13 @@
         <v>46314</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G9" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -1375,10 +1387,10 @@
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G10" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -1401,10 +1413,10 @@
         <v>6</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G11" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -1427,16 +1439,13 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
-        <v>12</v>
-      </c>
       <c r="B13" s="3">
         <f t="shared" si="2"/>
         <v>46342</v>
@@ -1450,7 +1459,7 @@
         <v>46342</v>
       </c>
       <c r="E13" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1467,12 +1476,12 @@
         <v>46349</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="3">
         <f t="shared" si="2"/>
@@ -1490,15 +1499,15 @@
         <v>8</v>
       </c>
       <c r="F15" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="G15" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="3">
         <f t="shared" si="2"/>
@@ -1519,12 +1528,12 @@
         <v>32</v>
       </c>
       <c r="G16" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="3">
         <f>B16+7</f>
@@ -1542,7 +1551,7 @@
         <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>